<commit_message>
Map Lead Reviewer names to initials in Column L
Use a lookup table of full names to initials for Column L instead of
full names, with alias fallbacks (first+middle, first+surname) for
names that appear shortened in the ExportMailAll data. Applied to
both the Python test script and the HTML app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7r88DkwB8DLxHVaDJntwG
</commit_message>
<xml_diff>
--- a/output_transmittal_register.xlsx
+++ b/output_transmittal_register.xlsx
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 17/06/2026 08:08</t>
+          <t>Generated: 17/06/2026 08:41</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Yazan Safieh</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="L53" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M53" s="4" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr"/>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M56" s="4" t="inlineStr">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M57" s="4" t="inlineStr"/>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M58" s="4" t="inlineStr"/>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M59" s="4" t="inlineStr"/>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M60" s="4" t="inlineStr">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="L61" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M61" s="4" t="inlineStr"/>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="L62" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M62" s="4" t="inlineStr"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M63" s="4" t="inlineStr"/>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="L64" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M64" s="4" t="inlineStr"/>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
-          <t>Amit Kumar</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="M65" s="4" t="inlineStr"/>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>Amit Kumar</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="M66" s="4" t="inlineStr"/>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="L67" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M67" s="4" t="inlineStr"/>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M68" s="4" t="inlineStr"/>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M69" s="4" t="inlineStr"/>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="L70" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M70" s="4" t="inlineStr"/>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M71" s="4" t="inlineStr"/>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>Ahmad Chikh bakri</t>
+          <t>ACB</t>
         </is>
       </c>
       <c r="M73" s="4" t="inlineStr"/>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="L74" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M74" s="4" t="inlineStr"/>
@@ -4769,7 +4769,7 @@
       </c>
       <c r="L75" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M75" s="4" t="inlineStr"/>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="L76" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M76" s="4" t="inlineStr"/>
@@ -4897,7 +4897,7 @@
       </c>
       <c r="L77" s="4" t="inlineStr">
         <is>
-          <t>Mohamed Yahia</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="M77" s="4" t="inlineStr"/>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="L78" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M78" s="4" t="inlineStr"/>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="L79" s="4" t="inlineStr">
         <is>
-          <t>Ahmad Chikh bakri</t>
+          <t>ACB</t>
         </is>
       </c>
       <c r="M79" s="4" t="inlineStr"/>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="L80" s="4" t="inlineStr">
         <is>
-          <t>Ahmad Chikh bakri</t>
+          <t>ACB</t>
         </is>
       </c>
       <c r="M80" s="4" t="inlineStr"/>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="L81" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M81" s="4" t="inlineStr"/>
@@ -5205,7 +5205,7 @@
       </c>
       <c r="L82" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M82" s="4" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L83" s="4" t="inlineStr">
         <is>
-          <t>Loren Leiski</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="M83" s="4" t="inlineStr"/>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="L84" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M84" s="4" t="inlineStr"/>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="L85" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M85" s="4" t="inlineStr"/>
@@ -5453,7 +5453,7 @@
       </c>
       <c r="L86" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M86" s="4" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="L87" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M87" s="4" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M88" s="4" t="inlineStr"/>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="L89" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M89" s="4" t="inlineStr"/>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M90" s="4" t="inlineStr"/>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="L91" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M91" s="4" t="inlineStr"/>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="L92" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M92" s="4" t="inlineStr"/>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M93" s="4" t="inlineStr"/>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="L94" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M94" s="4" t="inlineStr"/>
@@ -6025,7 +6025,7 @@
       </c>
       <c r="L95" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M95" s="4" t="inlineStr"/>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="L96" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M96" s="4" t="inlineStr"/>
@@ -6153,7 +6153,7 @@
       </c>
       <c r="L97" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M97" s="4" t="inlineStr"/>
@@ -6205,7 +6205,7 @@
       </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M98" s="4" t="inlineStr">
@@ -6261,7 +6261,7 @@
       </c>
       <c r="L99" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M99" s="4" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="L100" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M100" s="4" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="L101" s="4" t="inlineStr">
         <is>
-          <t>John Prabhu</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="M101" s="4" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="L105" s="4" t="inlineStr">
         <is>
-          <t>John Prabhu</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="M105" s="4" t="inlineStr">
@@ -7009,7 +7009,7 @@
       </c>
       <c r="L111" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M111" s="4" t="inlineStr"/>
@@ -7061,7 +7061,7 @@
       </c>
       <c r="L112" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M112" s="4" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="L113" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M113" s="4" t="inlineStr"/>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="L115" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M115" s="4" t="inlineStr"/>
@@ -7305,7 +7305,7 @@
       </c>
       <c r="L116" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M116" s="4" t="inlineStr">
@@ -7361,7 +7361,7 @@
       </c>
       <c r="L117" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M117" s="4" t="inlineStr">
@@ -7413,7 +7413,7 @@
       </c>
       <c r="L118" s="4" t="inlineStr">
         <is>
-          <t>Mike Lewey</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="M118" s="4" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="L119" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M119" s="4" t="inlineStr"/>
@@ -7545,7 +7545,7 @@
       </c>
       <c r="L120" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M120" s="4" t="inlineStr"/>
@@ -7609,7 +7609,7 @@
       </c>
       <c r="L121" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M121" s="4" t="inlineStr"/>
@@ -7673,7 +7673,7 @@
       </c>
       <c r="L122" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M122" s="4" t="inlineStr"/>
@@ -7737,7 +7737,7 @@
       </c>
       <c r="L123" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M123" s="4" t="inlineStr"/>
@@ -7801,7 +7801,7 @@
       </c>
       <c r="L124" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M124" s="4" t="inlineStr"/>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="L125" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M125" s="4" t="inlineStr">
@@ -7901,7 +7901,7 @@
       </c>
       <c r="L126" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M126" s="4" t="inlineStr">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="L127" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M127" s="4" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="L128" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M128" s="4" t="inlineStr">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="L129" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M129" s="4" t="inlineStr"/>
@@ -8137,7 +8137,7 @@
       </c>
       <c r="L130" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M130" s="4" t="inlineStr"/>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="L131" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M131" s="4" t="inlineStr"/>
@@ -8265,7 +8265,7 @@
       </c>
       <c r="L132" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M132" s="4" t="inlineStr"/>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="L133" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M133" s="4" t="inlineStr"/>
@@ -8393,7 +8393,7 @@
       </c>
       <c r="L134" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M134" s="4" t="inlineStr"/>
@@ -8457,7 +8457,7 @@
       </c>
       <c r="L135" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M135" s="4" t="inlineStr"/>
@@ -8521,7 +8521,7 @@
       </c>
       <c r="L136" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M136" s="4" t="inlineStr"/>
@@ -8585,7 +8585,7 @@
       </c>
       <c r="L137" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M137" s="4" t="inlineStr"/>
@@ -8637,7 +8637,7 @@
       </c>
       <c r="L138" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M138" s="4" t="inlineStr"/>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="L139" s="4" t="inlineStr">
         <is>
-          <t>Loren Leiski</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="M139" s="4" t="inlineStr"/>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="L140" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M140" s="4" t="inlineStr">
@@ -8833,7 +8833,7 @@
       </c>
       <c r="L141" s="4" t="inlineStr">
         <is>
-          <t>Evripidis Zampiras</t>
+          <t>EZ</t>
         </is>
       </c>
       <c r="M141" s="4" t="inlineStr"/>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="L142" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M142" s="4" t="inlineStr">
@@ -8953,7 +8953,7 @@
       </c>
       <c r="L143" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M143" s="4" t="inlineStr"/>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="L144" s="4" t="inlineStr">
         <is>
-          <t>Mohsin Patel</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="M144" s="4" t="inlineStr"/>
@@ -9081,7 +9081,7 @@
       </c>
       <c r="L145" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M145" s="4" t="inlineStr"/>
@@ -9145,7 +9145,7 @@
       </c>
       <c r="L146" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M146" s="4" t="inlineStr"/>
@@ -9209,7 +9209,7 @@
       </c>
       <c r="L147" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M147" s="4" t="inlineStr"/>
@@ -9273,7 +9273,7 @@
       </c>
       <c r="L148" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M148" s="4" t="inlineStr"/>
@@ -9337,7 +9337,7 @@
       </c>
       <c r="L149" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M149" s="4" t="inlineStr"/>
@@ -9401,7 +9401,7 @@
       </c>
       <c r="L150" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M150" s="4" t="inlineStr"/>
@@ -9465,7 +9465,7 @@
       </c>
       <c r="L151" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M151" s="4" t="inlineStr"/>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="L152" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M152" s="4" t="inlineStr"/>
@@ -9593,7 +9593,7 @@
       </c>
       <c r="L153" s="4" t="inlineStr">
         <is>
-          <t>Mohsin Patel</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="M153" s="4" t="inlineStr"/>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="L154" s="4" t="inlineStr">
         <is>
-          <t>Mohsin Patel</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="M154" s="4" t="inlineStr"/>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="L155" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M155" s="4" t="inlineStr">
@@ -9795,7 +9795,7 @@
       </c>
       <c r="L156" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M156" s="4" t="inlineStr"/>
@@ -9859,7 +9859,7 @@
       </c>
       <c r="L157" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M157" s="4" t="inlineStr"/>
@@ -9923,7 +9923,7 @@
       </c>
       <c r="L158" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M158" s="4" t="inlineStr"/>
@@ -9987,7 +9987,7 @@
       </c>
       <c r="L159" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M159" s="4" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="L160" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M160" s="4" t="inlineStr"/>
@@ -10119,7 +10119,7 @@
       </c>
       <c r="L161" s="4" t="inlineStr">
         <is>
-          <t>Loren Leiski</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="M161" s="4" t="inlineStr"/>
@@ -10171,7 +10171,7 @@
       </c>
       <c r="L162" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M162" s="4" t="inlineStr">
@@ -10239,7 +10239,7 @@
       </c>
       <c r="L163" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M163" s="4" t="inlineStr"/>
@@ -10303,7 +10303,7 @@
       </c>
       <c r="L164" s="4" t="inlineStr">
         <is>
-          <t>Siddarth Jayaraman</t>
+          <t>SRJ</t>
         </is>
       </c>
       <c r="M164" s="4" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="L165" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M165" s="4" t="inlineStr">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="L166" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M166" s="4" t="inlineStr"/>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="L168" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M168" s="4" t="inlineStr">
@@ -10607,7 +10607,7 @@
       </c>
       <c r="L169" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M169" s="4" t="inlineStr"/>
@@ -10671,7 +10671,7 @@
       </c>
       <c r="L170" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M170" s="4" t="inlineStr"/>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="L171" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M171" s="4" t="inlineStr">
@@ -10873,7 +10873,7 @@
       </c>
       <c r="L173" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M173" s="4" t="inlineStr"/>
@@ -10937,7 +10937,7 @@
       </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M174" s="4" t="inlineStr"/>
@@ -11001,7 +11001,7 @@
       </c>
       <c r="L175" s="4" t="inlineStr">
         <is>
-          <t>Mohsin Patel</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="M175" s="4" t="inlineStr"/>
@@ -11053,7 +11053,7 @@
       </c>
       <c r="L176" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M176" s="4" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="L177" s="8" t="inlineStr">
         <is>
-          <t>Oladele Kupolati</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="M177" s="8" t="inlineStr"/>
@@ -11189,7 +11189,7 @@
       </c>
       <c r="L178" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M178" s="4" t="inlineStr"/>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="L179" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M179" s="4" t="inlineStr"/>
@@ -11317,7 +11317,7 @@
       </c>
       <c r="L180" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M180" s="4" t="inlineStr">
@@ -11385,7 +11385,7 @@
       </c>
       <c r="L181" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M181" s="4" t="inlineStr"/>
@@ -11449,7 +11449,7 @@
       </c>
       <c r="L182" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M182" s="4" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="L183" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M183" s="4" t="inlineStr"/>
@@ -11581,7 +11581,7 @@
       </c>
       <c r="L184" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M184" s="4" t="inlineStr"/>
@@ -11651,7 +11651,7 @@
       </c>
       <c r="L185" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M185" s="4" t="inlineStr"/>
@@ -11703,7 +11703,7 @@
       </c>
       <c r="L186" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M186" s="4" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="L187" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M187" s="4" t="inlineStr"/>
@@ -11841,7 +11841,7 @@
       </c>
       <c r="L188" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M188" s="4" t="inlineStr"/>
@@ -11911,7 +11911,7 @@
       </c>
       <c r="L189" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M189" s="4" t="inlineStr"/>
@@ -11975,7 +11975,7 @@
       </c>
       <c r="L190" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M190" s="4" t="inlineStr"/>
@@ -12027,7 +12027,7 @@
       </c>
       <c r="L191" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M191" s="4" t="inlineStr">
@@ -12095,7 +12095,7 @@
       </c>
       <c r="L192" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M192" s="4" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="L193" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M193" s="4" t="inlineStr">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="L194" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M194" s="4" t="inlineStr">
@@ -12287,7 +12287,7 @@
       </c>
       <c r="L195" s="4" t="inlineStr">
         <is>
-          <t>Evripidis Zampiras</t>
+          <t>EZ</t>
         </is>
       </c>
       <c r="M195" s="4" t="inlineStr"/>
@@ -12351,7 +12351,7 @@
       </c>
       <c r="L196" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M196" s="4" t="inlineStr"/>
@@ -12403,7 +12403,7 @@
       </c>
       <c r="L197" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M197" s="4" t="inlineStr">
@@ -12459,7 +12459,7 @@
       </c>
       <c r="L198" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M198" s="4" t="inlineStr">
@@ -12527,7 +12527,7 @@
       </c>
       <c r="L199" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M199" s="4" t="inlineStr"/>
@@ -12575,7 +12575,7 @@
       </c>
       <c r="L200" s="4" t="inlineStr">
         <is>
-          <t>Yazan Safieh</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M200" s="4" t="inlineStr">
@@ -12643,7 +12643,7 @@
       </c>
       <c r="L201" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M201" s="4" t="inlineStr"/>
@@ -12707,7 +12707,7 @@
       </c>
       <c r="L202" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M202" s="4" t="inlineStr"/>
@@ -12771,7 +12771,7 @@
       </c>
       <c r="L203" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M203" s="4" t="inlineStr"/>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="L204" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M204" s="4" t="inlineStr"/>
@@ -12899,7 +12899,7 @@
       </c>
       <c r="L205" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M205" s="4" t="inlineStr"/>
@@ -12963,7 +12963,7 @@
       </c>
       <c r="L206" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M206" s="4" t="inlineStr"/>
@@ -13027,7 +13027,7 @@
       </c>
       <c r="L207" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M207" s="4" t="inlineStr"/>
@@ -13097,7 +13097,7 @@
       </c>
       <c r="L208" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M208" s="4" t="inlineStr"/>
@@ -13167,7 +13167,7 @@
       </c>
       <c r="L209" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M209" s="4" t="inlineStr"/>
@@ -13231,7 +13231,7 @@
       </c>
       <c r="L210" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M210" s="4" t="inlineStr"/>
@@ -13295,7 +13295,7 @@
       </c>
       <c r="L211" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M211" s="4" t="inlineStr"/>
@@ -13365,7 +13365,7 @@
       </c>
       <c r="L212" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M212" s="4" t="inlineStr">
@@ -13439,7 +13439,7 @@
       </c>
       <c r="L213" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M213" s="4" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="L214" s="4" t="inlineStr">
         <is>
-          <t>Kaddour Lardjani</t>
+          <t>KLI</t>
         </is>
       </c>
       <c r="M214" s="4" t="inlineStr"/>
@@ -13559,7 +13559,7 @@
       </c>
       <c r="L215" s="4" t="inlineStr">
         <is>
-          <t>Daniel Maddy</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="M215" s="4" t="inlineStr">
@@ -13615,7 +13615,7 @@
       </c>
       <c r="L216" s="4" t="inlineStr">
         <is>
-          <t>Sandeep Jha</t>
+          <t>SJ</t>
         </is>
       </c>
       <c r="M216" s="4" t="inlineStr">
@@ -13667,7 +13667,7 @@
       </c>
       <c r="L217" s="4" t="inlineStr">
         <is>
-          <t>Sandeep Jha</t>
+          <t>SJ</t>
         </is>
       </c>
       <c r="M217" s="4" t="inlineStr">
@@ -14231,7 +14231,7 @@
       </c>
       <c r="L226" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M226" s="4" t="inlineStr"/>
@@ -14295,7 +14295,7 @@
       </c>
       <c r="L227" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M227" s="4" t="inlineStr"/>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="L228" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M228" s="4" t="inlineStr"/>
@@ -14423,7 +14423,7 @@
       </c>
       <c r="L229" s="4" t="inlineStr">
         <is>
-          <t>Ahmad Chikh bakri</t>
+          <t>ACB</t>
         </is>
       </c>
       <c r="M229" s="4" t="inlineStr"/>
@@ -14487,7 +14487,7 @@
       </c>
       <c r="L230" s="4" t="inlineStr">
         <is>
-          <t>Allan Halferty</t>
+          <t>AH</t>
         </is>
       </c>
       <c r="M230" s="4" t="inlineStr"/>
@@ -14551,7 +14551,7 @@
       </c>
       <c r="L231" s="4" t="inlineStr">
         <is>
-          <t>Nageswara Ampolu</t>
+          <t>NRA</t>
         </is>
       </c>
       <c r="M231" s="4" t="inlineStr"/>
@@ -14615,7 +14615,7 @@
       </c>
       <c r="L232" s="4" t="inlineStr">
         <is>
-          <t>John Prabhu</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="M232" s="4" t="inlineStr"/>
@@ -14679,7 +14679,7 @@
       </c>
       <c r="L233" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M233" s="4" t="inlineStr"/>
@@ -14731,7 +14731,7 @@
       </c>
       <c r="L234" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M234" s="4" t="inlineStr">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="L235" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M235" s="4" t="inlineStr"/>
@@ -14851,7 +14851,7 @@
       </c>
       <c r="L236" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M236" s="4" t="inlineStr"/>
@@ -14915,7 +14915,7 @@
       </c>
       <c r="L237" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M237" s="4" t="inlineStr"/>
@@ -14979,7 +14979,7 @@
       </c>
       <c r="L238" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M238" s="4" t="inlineStr"/>
@@ -15043,7 +15043,7 @@
       </c>
       <c r="L239" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M239" s="4" t="inlineStr"/>
@@ -15107,7 +15107,7 @@
       </c>
       <c r="L240" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M240" s="4" t="inlineStr"/>
@@ -15171,7 +15171,7 @@
       </c>
       <c r="L241" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M241" s="4" t="inlineStr"/>
@@ -15235,7 +15235,7 @@
       </c>
       <c r="L242" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M242" s="4" t="inlineStr"/>
@@ -15299,7 +15299,7 @@
       </c>
       <c r="L243" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M243" s="4" t="inlineStr"/>
@@ -15363,7 +15363,7 @@
       </c>
       <c r="L244" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M244" s="4" t="inlineStr"/>
@@ -15427,7 +15427,7 @@
       </c>
       <c r="L245" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M245" s="4" t="inlineStr"/>
@@ -15491,7 +15491,7 @@
       </c>
       <c r="L246" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M246" s="4" t="inlineStr"/>
@@ -15543,7 +15543,7 @@
       </c>
       <c r="L247" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M247" s="4" t="inlineStr">
@@ -15611,7 +15611,7 @@
       </c>
       <c r="L248" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M248" s="4" t="inlineStr"/>
@@ -15681,7 +15681,7 @@
       </c>
       <c r="L249" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M249" s="4" t="inlineStr"/>
@@ -15811,7 +15811,7 @@
       </c>
       <c r="L251" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M251" s="4" t="inlineStr"/>
@@ -15875,7 +15875,7 @@
       </c>
       <c r="L252" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M252" s="4" t="inlineStr"/>
@@ -15939,7 +15939,7 @@
       </c>
       <c r="L253" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M253" s="4" t="inlineStr"/>
@@ -16003,7 +16003,7 @@
       </c>
       <c r="L254" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M254" s="4" t="inlineStr"/>
@@ -16055,7 +16055,7 @@
       </c>
       <c r="L255" s="4" t="inlineStr">
         <is>
-          <t>Yazan Safieh</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M255" s="4" t="inlineStr">
@@ -16107,7 +16107,7 @@
       </c>
       <c r="L256" s="4" t="inlineStr">
         <is>
-          <t>Yazan Safieh</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M256" s="4" t="inlineStr">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="L257" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M257" s="4" t="inlineStr">
@@ -16231,7 +16231,7 @@
       </c>
       <c r="L258" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M258" s="4" t="inlineStr"/>
@@ -16283,7 +16283,7 @@
       </c>
       <c r="L259" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M259" s="4" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="L260" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M260" s="4" t="inlineStr"/>
@@ -16415,7 +16415,7 @@
       </c>
       <c r="L261" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M261" s="4" t="inlineStr"/>
@@ -16467,7 +16467,7 @@
       </c>
       <c r="L262" s="4" t="inlineStr">
         <is>
-          <t>Ashok Kumar</t>
+          <t>AKM</t>
         </is>
       </c>
       <c r="M262" s="4" t="inlineStr"/>
@@ -16525,7 +16525,7 @@
       </c>
       <c r="L263" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M263" s="4" t="inlineStr">
@@ -16593,7 +16593,7 @@
       </c>
       <c r="L264" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M264" s="4" t="inlineStr"/>
@@ -16663,7 +16663,7 @@
       </c>
       <c r="L265" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M265" s="4" t="inlineStr"/>
@@ -16733,7 +16733,7 @@
       </c>
       <c r="L266" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M266" s="4" t="inlineStr"/>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="L267" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M267" s="4" t="inlineStr"/>
@@ -16861,7 +16861,7 @@
       </c>
       <c r="L268" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M268" s="4" t="inlineStr"/>
@@ -16925,7 +16925,7 @@
       </c>
       <c r="L269" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M269" s="4" t="inlineStr">
@@ -16993,7 +16993,7 @@
       </c>
       <c r="L270" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M270" s="4" t="inlineStr">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="L271" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M271" s="4" t="inlineStr">
@@ -17129,7 +17129,7 @@
       </c>
       <c r="L272" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M272" s="4" t="inlineStr">
@@ -17197,7 +17197,7 @@
       </c>
       <c r="L273" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M273" s="4" t="inlineStr">
@@ -17265,7 +17265,7 @@
       </c>
       <c r="L274" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M274" s="4" t="inlineStr"/>
@@ -17317,7 +17317,7 @@
       </c>
       <c r="L275" s="4" t="inlineStr">
         <is>
-          <t>Mike Lewey</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="M275" s="4" t="inlineStr">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="L276" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M276" s="4" t="inlineStr"/>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="L277" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M277" s="4" t="inlineStr">
@@ -17505,7 +17505,7 @@
       </c>
       <c r="L278" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M278" s="4" t="inlineStr"/>
@@ -17569,7 +17569,7 @@
       </c>
       <c r="L279" s="4" t="inlineStr">
         <is>
-          <t>Mohamed Yahia</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="M279" s="4" t="inlineStr"/>
@@ -17633,7 +17633,7 @@
       </c>
       <c r="L280" s="4" t="inlineStr">
         <is>
-          <t>Stephen Beadle</t>
+          <t>SAB</t>
         </is>
       </c>
       <c r="M280" s="4" t="inlineStr"/>
@@ -17697,7 +17697,7 @@
       </c>
       <c r="L281" s="4" t="inlineStr">
         <is>
-          <t>Nageswara Ampolu</t>
+          <t>NRA</t>
         </is>
       </c>
       <c r="M281" s="4" t="inlineStr"/>
@@ -17761,7 +17761,7 @@
       </c>
       <c r="L282" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M282" s="4" t="inlineStr"/>
@@ -17825,7 +17825,7 @@
       </c>
       <c r="L283" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M283" s="4" t="inlineStr"/>
@@ -17889,7 +17889,7 @@
       </c>
       <c r="L284" s="4" t="inlineStr">
         <is>
-          <t>Amit Kumar</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="M284" s="4" t="inlineStr"/>
@@ -17947,7 +17947,7 @@
       </c>
       <c r="L285" s="4" t="inlineStr">
         <is>
-          <t>Amit Kumar</t>
+          <t>AK</t>
         </is>
       </c>
       <c r="M285" s="4" t="inlineStr"/>
@@ -18011,7 +18011,7 @@
       </c>
       <c r="L286" s="4" t="inlineStr">
         <is>
-          <t>Alister White</t>
+          <t>AW</t>
         </is>
       </c>
       <c r="M286" s="4" t="inlineStr"/>
@@ -18075,7 +18075,7 @@
       </c>
       <c r="L287" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M287" s="4" t="inlineStr"/>
@@ -18139,7 +18139,7 @@
       </c>
       <c r="L288" s="4" t="inlineStr">
         <is>
-          <t>Loren Leiski</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="M288" s="4" t="inlineStr"/>
@@ -18203,7 +18203,7 @@
       </c>
       <c r="L289" s="4" t="inlineStr">
         <is>
-          <t>Loren Leiski</t>
+          <t>LL</t>
         </is>
       </c>
       <c r="M289" s="4" t="inlineStr"/>
@@ -18251,7 +18251,7 @@
       </c>
       <c r="L290" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M290" s="4" t="inlineStr"/>
@@ -18315,7 +18315,7 @@
       </c>
       <c r="L291" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M291" s="4" t="inlineStr"/>
@@ -18379,7 +18379,7 @@
       </c>
       <c r="L292" s="4" t="inlineStr">
         <is>
-          <t>Ahmad Chikh bakri</t>
+          <t>ACB</t>
         </is>
       </c>
       <c r="M292" s="4" t="inlineStr"/>
@@ -18443,7 +18443,7 @@
       </c>
       <c r="L293" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M293" s="4" t="inlineStr"/>
@@ -18503,7 +18503,7 @@
       </c>
       <c r="L294" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M294" s="4" t="inlineStr"/>
@@ -18567,7 +18567,7 @@
       </c>
       <c r="L295" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M295" s="4" t="inlineStr"/>
@@ -18637,7 +18637,7 @@
       </c>
       <c r="L296" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M296" s="4" t="inlineStr"/>
@@ -18701,7 +18701,7 @@
       </c>
       <c r="L297" s="4" t="inlineStr">
         <is>
-          <t>Lynneth Santos</t>
+          <t>LS</t>
         </is>
       </c>
       <c r="M297" s="4" t="inlineStr"/>
@@ -18765,7 +18765,7 @@
       </c>
       <c r="L298" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M298" s="4" t="inlineStr"/>
@@ -18829,7 +18829,7 @@
       </c>
       <c r="L299" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M299" s="4" t="inlineStr"/>
@@ -18893,7 +18893,7 @@
       </c>
       <c r="L300" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M300" s="4" t="inlineStr">
@@ -18967,7 +18967,7 @@
       </c>
       <c r="L301" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M301" s="4" t="inlineStr"/>
@@ -19037,7 +19037,7 @@
       </c>
       <c r="L302" s="4" t="inlineStr">
         <is>
-          <t>Arunkumar Ramakrishnan</t>
+          <t>AKR</t>
         </is>
       </c>
       <c r="M302" s="4" t="inlineStr"/>
@@ -19101,7 +19101,7 @@
       </c>
       <c r="L303" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M303" s="4" t="inlineStr"/>
@@ -19153,7 +19153,7 @@
       </c>
       <c r="L304" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M304" s="4" t="inlineStr">
@@ -19221,7 +19221,7 @@
       </c>
       <c r="L305" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M305" s="4" t="inlineStr"/>
@@ -19291,7 +19291,7 @@
       </c>
       <c r="L306" s="4" t="inlineStr">
         <is>
-          <t>Rohit Tharakan</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="M306" s="4" t="inlineStr">
@@ -19359,7 +19359,7 @@
       </c>
       <c r="L307" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M307" s="4" t="inlineStr"/>
@@ -19411,7 +19411,7 @@
       </c>
       <c r="L308" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M308" s="4" t="inlineStr">
@@ -19601,7 +19601,7 @@
       </c>
       <c r="L311" s="4" t="inlineStr">
         <is>
-          <t>Vinod Kalwaghe</t>
+          <t>VAK</t>
         </is>
       </c>
       <c r="M311" s="4" t="inlineStr"/>
@@ -19801,7 +19801,7 @@
       </c>
       <c r="L314" s="4" t="inlineStr">
         <is>
-          <t>Mohsin Patel</t>
+          <t>MP</t>
         </is>
       </c>
       <c r="M314" s="4" t="inlineStr"/>
@@ -19859,7 +19859,7 @@
       </c>
       <c r="L315" s="4" t="inlineStr">
         <is>
-          <t>Mike Lewey</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="M315" s="4" t="inlineStr">
@@ -19927,7 +19927,7 @@
       </c>
       <c r="L316" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M316" s="4" t="inlineStr"/>
@@ -19991,7 +19991,7 @@
       </c>
       <c r="L317" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M317" s="4" t="inlineStr"/>
@@ -20055,7 +20055,7 @@
       </c>
       <c r="L318" s="4" t="inlineStr">
         <is>
-          <t>Mazar Syed</t>
+          <t>MSD</t>
         </is>
       </c>
       <c r="M318" s="4" t="inlineStr"/>
@@ -20107,7 +20107,7 @@
       </c>
       <c r="L319" s="4" t="inlineStr">
         <is>
-          <t>Yazan Safieh</t>
+          <t>YS</t>
         </is>
       </c>
       <c r="M319" s="4" t="inlineStr">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="L320" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M320" s="4" t="inlineStr">
@@ -20223,7 +20223,7 @@
       </c>
       <c r="L321" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M321" s="4" t="inlineStr">
@@ -20275,7 +20275,7 @@
       </c>
       <c r="L322" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M322" s="4" t="inlineStr">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="L323" s="4" t="inlineStr">
         <is>
-          <t>Sherif Zayed</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M323" s="4" t="inlineStr">
@@ -20465,7 +20465,7 @@
       </c>
       <c r="L325" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M325" s="4" t="inlineStr"/>
@@ -20529,7 +20529,7 @@
       </c>
       <c r="L326" s="4" t="inlineStr">
         <is>
-          <t>Alister White</t>
+          <t>AW</t>
         </is>
       </c>
       <c r="M326" s="4" t="inlineStr"/>
@@ -20593,7 +20593,7 @@
       </c>
       <c r="L327" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M327" s="4" t="inlineStr">
@@ -20661,7 +20661,7 @@
       </c>
       <c r="L328" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M328" s="4" t="inlineStr"/>
@@ -20725,7 +20725,7 @@
       </c>
       <c r="L329" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M329" s="4" t="inlineStr"/>
@@ -20789,7 +20789,7 @@
       </c>
       <c r="L330" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M330" s="4" t="inlineStr"/>
@@ -20853,7 +20853,7 @@
       </c>
       <c r="L331" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M331" s="4" t="inlineStr"/>
@@ -20917,7 +20917,7 @@
       </c>
       <c r="L332" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M332" s="4" t="inlineStr"/>
@@ -20981,7 +20981,7 @@
       </c>
       <c r="L333" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M333" s="4" t="inlineStr"/>
@@ -21045,7 +21045,7 @@
       </c>
       <c r="L334" s="4" t="inlineStr">
         <is>
-          <t>Ahmed Ibrahim</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="M334" s="4" t="inlineStr"/>
@@ -21109,7 +21109,7 @@
       </c>
       <c r="L335" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M335" s="4" t="inlineStr"/>
@@ -21173,7 +21173,7 @@
       </c>
       <c r="L336" s="4" t="inlineStr">
         <is>
-          <t>Ismaiel Salama</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="M336" s="4" t="inlineStr"/>
@@ -21237,7 +21237,7 @@
       </c>
       <c r="L337" s="4" t="inlineStr">
         <is>
-          <t>Suresh Shetty</t>
+          <t>SSY</t>
         </is>
       </c>
       <c r="M337" s="4" t="inlineStr"/>
@@ -21347,7 +21347,7 @@
       </c>
       <c r="L339" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M339" s="4" t="inlineStr">
@@ -21415,7 +21415,7 @@
       </c>
       <c r="L340" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M340" s="4" t="inlineStr"/>
@@ -21479,7 +21479,7 @@
       </c>
       <c r="L341" s="4" t="inlineStr">
         <is>
-          <t>Shahab Ahmad Khan</t>
+          <t>SAK</t>
         </is>
       </c>
       <c r="M341" s="4" t="inlineStr"/>
@@ -21543,7 +21543,7 @@
       </c>
       <c r="L342" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M342" s="4" t="inlineStr">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="L343" s="4" t="inlineStr">
         <is>
-          <t>Mahmoud Saad</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="M343" s="4" t="inlineStr">
@@ -46607,7 +46607,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>17/06/2026 08:08</t>
+          <t>17/06/2026 08:41</t>
         </is>
       </c>
     </row>

</xml_diff>